<commit_message>
feat: projeto mca loan
</commit_message>
<xml_diff>
--- a/MCA_Final_Report.xlsx
+++ b/MCA_Final_Report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX8"/>
+  <dimension ref="A1:AX9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1853,10 +1853,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>0000007372</t>
-        </is>
+      <c r="A8" t="n">
+        <v>7372</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
@@ -1894,10 +1892,8 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>000000737277969</t>
-        </is>
+      <c r="N8" t="n">
+        <v>737277969</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
@@ -2059,6 +2055,218 @@
         </is>
       </c>
       <c r="AX8" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>0000007372</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ABUNDANCE E-COMMERCE LLC International Calls: 1-713-262-1679</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2804 TIMBERBROOK DR We accept operator relay calls</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>CHARLOTTE</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>28208-3323</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>000000737277969</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>$5,000.00</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 3,372.00</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 3,000.00</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 3,394.00</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 7,500.00</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 2,000.00</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 3,661.00</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1,000.00</t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 5,000.00</t>
+        </is>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AW9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 3,813.00</t>
+        </is>
+      </c>
+      <c r="AX9" t="inlineStr">
         <is>
           <t>Found in statement</t>
         </is>

</xml_diff>

<commit_message>
fix: :bug: resolvido readme atualizado para cliente americanos
</commit_message>
<xml_diff>
--- a/MCA_Final_Report.xlsx
+++ b/MCA_Final_Report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX9"/>
+  <dimension ref="A1:AX11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2061,10 +2061,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>0000007372</t>
-        </is>
+      <c r="A9" t="n">
+        <v>7372</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
@@ -2102,10 +2100,8 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>000000737277969</t>
-        </is>
+      <c r="N9" t="n">
+        <v>737277969</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
@@ -2267,6 +2263,430 @@
         </is>
       </c>
       <c r="AX9" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0000007372</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ABUNDANCE E-COMMERCE LLC International Calls: 1-713-262-1679</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2804 TIMBERBROOK DR We accept operator relay calls</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>CHARLOTTE</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>28208-3323</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>000000737277969</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>$2,849.00</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 5,000.00</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 5,000.00</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 2,726.00</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 110.00</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 5,000.00</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 4,999.00</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 5,000.00</t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1,250.00</t>
+        </is>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 400.00</t>
+        </is>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0000007372</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ABUNDANCE E-COMMERCE LLC International Calls: 1-713-262-1679</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2804 TIMBERBROOK DR We accept operator relay calls</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>CHARLOTTE</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>28208-3323</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>000000737277969</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>$3,430.00</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 5,000.00</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 310.69</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 5,000.00</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 3,440.00</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 3,350.00</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 3,500.00</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1,750.00</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 250.00</t>
+        </is>
+      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>Found in statement</t>
+        </is>
+      </c>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AW11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 250.00</t>
+        </is>
+      </c>
+      <c r="AX11" t="inlineStr">
         <is>
           <t>Found in statement</t>
         </is>

</xml_diff>